<commit_message>
day 15 aws deployment methods and  xg boost learning docs
</commit_message>
<xml_diff>
--- a/AWS ML Specialization/4_Model_Performance_Evaluation/HoursExamSample_ConfusionMatrix_Worksheet_3.xlsx
+++ b/AWS ML Specialization/4_Model_Performance_Evaluation/HoursExamSample_ConfusionMatrix_Worksheet_3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AWSMLSageMaker\201906\VideoScripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Data_Science\Machine-Learning-Projects\AWS ML Specialization\4_Model_Performance_Evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEC0408-0E50-402B-8AF0-14F281A59E16}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9C40B8-4473-4B81-9AEF-C58316EDA216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1725" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HoursExamSample_ConfusionMatrix" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -718,9 +723,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -758,7 +763,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -864,7 +869,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1006,7 +1011,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1015,17 +1020,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" customWidth="1"/>
-    <col min="2" max="2" width="6.6328125" customWidth="1"/>
-    <col min="3" max="3" width="18.54296875" customWidth="1"/>
-    <col min="5" max="5" width="19.90625" customWidth="1"/>
-    <col min="8" max="8" width="9.453125" customWidth="1"/>
-    <col min="9" max="9" width="23.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.21875" customWidth="1"/>
+    <col min="2" max="2" width="6.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" customWidth="1"/>
+    <col min="8" max="8" width="9.44140625" customWidth="1"/>
+    <col min="9" max="9" width="23.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1039,7 +1044,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0.5</v>
       </c>
@@ -1059,7 +1064,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0.75</v>
       </c>
@@ -1079,7 +1084,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1090,7 +1095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1.25</v>
       </c>
@@ -1110,7 +1115,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1.5</v>
       </c>
@@ -1130,7 +1135,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1.75</v>
       </c>
@@ -1141,7 +1146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1.75</v>
       </c>
@@ -1155,7 +1160,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1170,7 +1175,7 @@
       </c>
       <c r="H9" s="6"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2.25</v>
       </c>
@@ -1187,7 +1192,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2.5</v>
       </c>
@@ -1214,7 +1219,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2.75</v>
       </c>
@@ -1239,7 +1244,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>3</v>
       </c>
@@ -1258,7 +1263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>3.25</v>
       </c>
@@ -1269,7 +1274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>3.5</v>
       </c>
@@ -1283,7 +1288,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>4</v>
       </c>
@@ -1298,7 +1303,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>4.25</v>
       </c>
@@ -1315,7 +1320,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4.5</v>
       </c>
@@ -1340,7 +1345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>4.75</v>
       </c>
@@ -1363,7 +1368,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>5</v>
       </c>
@@ -1374,7 +1379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>5.5</v>
       </c>
@@ -1402,15 +1407,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="C3:J15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="9" max="9" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
         <v>20</v>
       </c>
@@ -1421,7 +1426,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>16</v>
       </c>
@@ -1441,7 +1446,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C5">
         <v>0</v>
       </c>
@@ -1461,7 +1466,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C6">
         <v>0.1</v>
       </c>
@@ -1481,7 +1486,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C7">
         <v>0.2</v>
       </c>
@@ -1501,7 +1506,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C8">
         <v>0.3</v>
       </c>
@@ -1521,7 +1526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C9">
         <v>0.4</v>
       </c>
@@ -1541,7 +1546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C10">
         <v>0.5</v>
       </c>
@@ -1561,7 +1566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C11">
         <v>0.6</v>
       </c>
@@ -1581,7 +1586,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C12">
         <v>0.7</v>
       </c>
@@ -1601,7 +1606,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C13">
         <v>0.8</v>
       </c>
@@ -1621,7 +1626,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C14">
         <v>0.9</v>
       </c>
@@ -1641,7 +1646,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C15">
         <v>1</v>
       </c>

</xml_diff>